<commit_message>
busca_fazenda: add busca multipla por fazendas
</commit_message>
<xml_diff>
--- a/datas_remessas.xlsx
+++ b/datas_remessas.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://agroroboticafca-my.sharepoint.com/personal/miguel_santos_agrorobotica_com_br/Documents/AGROROBOTICA/PROJETOS/Dashoboard_ATVOS/datas_remessas/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://agroroboticafca-my.sharepoint.com/personal/miguel_santos_agrorobotica_com_br/Documents/AGROROBOTICA/PROJETOS/Dashoboard_ATVOS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="384" documentId="11_F25DC773A252ABDACC10489B791D7F6E5BDE58EE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EFD04C38-E0E0-4380-8CB2-8E22DDA2E1C8}"/>
+  <xr:revisionPtr revIDLastSave="390" documentId="11_F25DC773A252ABDACC10489B791D7F6E5BDE58EE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{869C961F-7640-4CBB-9B99-0C75C89211B5}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -165,7 +165,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.59999389629810485"/>
+        <fgColor theme="4" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -182,7 +182,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -193,13 +193,16 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -497,22 +500,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="4" t="s">
         <v>33</v>
       </c>
     </row>
@@ -580,169 +583,169 @@
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="C5" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="D5" s="6">
+      <c r="C5" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="D5" s="7">
         <v>46146</v>
       </c>
-      <c r="E5" s="6">
-        <v>46156</v>
-      </c>
-      <c r="F5" s="1" t="str">
+      <c r="E5" s="7">
+        <v>46148</v>
+      </c>
+      <c r="F5" s="6" t="str">
         <f t="shared" si="0"/>
         <v>Concluído</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="C6" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="D6" s="6">
+      <c r="C6" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="D6" s="7">
         <v>46146</v>
       </c>
-      <c r="E6" s="6">
-        <v>46156</v>
-      </c>
-      <c r="F6" s="1" t="str">
+      <c r="E6" s="7">
+        <v>46148</v>
+      </c>
+      <c r="F6" s="6" t="str">
         <f t="shared" si="0"/>
         <v>Concluído</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="C7" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="D7" s="3">
+      <c r="C7" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="D7" s="7">
         <v>46146</v>
       </c>
-      <c r="E7" s="3">
+      <c r="E7" s="7">
         <v>46149</v>
       </c>
-      <c r="F7" s="1" t="str">
+      <c r="F7" s="6" t="str">
         <f t="shared" si="0"/>
         <v>Concluído</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="C8" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="D8" s="6">
+      <c r="C8" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8" s="7">
         <v>46146</v>
       </c>
-      <c r="E8" s="6">
-        <v>46156</v>
-      </c>
-      <c r="F8" s="1" t="str">
+      <c r="E8" s="7">
+        <v>46148</v>
+      </c>
+      <c r="F8" s="6" t="str">
         <f t="shared" si="0"/>
         <v>Concluído</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
+      <c r="A9" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="C9" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="D9" s="3">
+      <c r="C9" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="D9" s="7">
         <v>46146</v>
       </c>
-      <c r="E9" s="3">
+      <c r="E9" s="7">
         <v>46149</v>
       </c>
-      <c r="F9" s="1" t="str">
+      <c r="F9" s="6" t="str">
         <f t="shared" si="0"/>
         <v>Concluído</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="4" t="s">
+      <c r="A10" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="C10" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="D10" s="6">
+      <c r="C10" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="D10" s="7">
         <v>46146</v>
       </c>
-      <c r="E10" s="6">
-        <v>46156</v>
-      </c>
-      <c r="F10" s="1" t="str">
+      <c r="E10" s="7">
+        <v>46148</v>
+      </c>
+      <c r="F10" s="6" t="str">
         <f t="shared" si="0"/>
         <v>Concluído</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
+      <c r="A11" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="C11" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="D11" s="3">
+      <c r="C11" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="D11" s="7">
         <v>46146</v>
       </c>
-      <c r="E11" s="3">
+      <c r="E11" s="7">
         <v>46149</v>
       </c>
-      <c r="F11" s="1" t="str">
+      <c r="F11" s="6" t="str">
         <f t="shared" si="0"/>
         <v>Concluído</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" s="4" t="s">
+      <c r="A12" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="C12" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="D12" s="6">
+      <c r="C12" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="D12" s="7">
         <v>46146</v>
       </c>
-      <c r="E12" s="6">
-        <v>46156</v>
-      </c>
-      <c r="F12" s="1" t="str">
+      <c r="E12" s="7">
+        <v>46148</v>
+      </c>
+      <c r="F12" s="6" t="str">
         <f t="shared" si="0"/>
         <v>Concluído</v>
       </c>

</xml_diff>

<commit_message>
adicao de data de entrega os 015, att st
</commit_message>
<xml_diff>
--- a/datas_remessas.xlsx
+++ b/datas_remessas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://agroroboticafca-my.sharepoint.com/personal/miguel_santos_agrorobotica_com_br/Documents/AGROROBOTICA/PROJETOS/Dashoboard_ATVOS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="390" documentId="11_F25DC773A252ABDACC10489B791D7F6E5BDE58EE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{869C961F-7640-4CBB-9B99-0C75C89211B5}"/>
+  <xr:revisionPtr revIDLastSave="392" documentId="11_F25DC773A252ABDACC10489B791D7F6E5BDE58EE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BEE64007-3303-4136-B7F0-609B7B639BD6}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="35">
   <si>
     <t>Remessa</t>
   </si>
@@ -182,7 +182,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -194,15 +194,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -583,169 +574,169 @@
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="C5" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="D5" s="7">
+      <c r="C5" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D5" s="3">
         <v>46146</v>
       </c>
-      <c r="E5" s="7">
+      <c r="E5" s="3">
         <v>46148</v>
       </c>
-      <c r="F5" s="6" t="str">
+      <c r="F5" s="1" t="str">
         <f t="shared" si="0"/>
         <v>Concluído</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C6" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="D6" s="7">
+      <c r="C6" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D6" s="3">
         <v>46146</v>
       </c>
-      <c r="E6" s="7">
+      <c r="E6" s="3">
         <v>46148</v>
       </c>
-      <c r="F6" s="6" t="str">
+      <c r="F6" s="1" t="str">
         <f t="shared" si="0"/>
         <v>Concluído</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C7" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="D7" s="7">
+      <c r="C7" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D7" s="3">
         <v>46146</v>
       </c>
-      <c r="E7" s="7">
+      <c r="E7" s="3">
         <v>46149</v>
       </c>
-      <c r="F7" s="6" t="str">
+      <c r="F7" s="1" t="str">
         <f t="shared" si="0"/>
         <v>Concluído</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="C8" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="D8" s="7">
+      <c r="C8" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8" s="3">
         <v>46146</v>
       </c>
-      <c r="E8" s="7">
+      <c r="E8" s="3">
         <v>46148</v>
       </c>
-      <c r="F8" s="6" t="str">
+      <c r="F8" s="1" t="str">
         <f t="shared" si="0"/>
         <v>Concluído</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="5" t="s">
+      <c r="A9" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="C9" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="D9" s="7">
+      <c r="C9" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D9" s="3">
         <v>46146</v>
       </c>
-      <c r="E9" s="7">
+      <c r="E9" s="3">
         <v>46149</v>
       </c>
-      <c r="F9" s="6" t="str">
+      <c r="F9" s="1" t="str">
         <f t="shared" si="0"/>
         <v>Concluído</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="5" t="s">
+      <c r="A10" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C10" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="D10" s="7">
+      <c r="C10" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D10" s="3">
         <v>46146</v>
       </c>
-      <c r="E10" s="7">
+      <c r="E10" s="3">
         <v>46148</v>
       </c>
-      <c r="F10" s="6" t="str">
+      <c r="F10" s="1" t="str">
         <f t="shared" si="0"/>
         <v>Concluído</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" s="5" t="s">
+      <c r="A11" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C11" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="D11" s="7">
+      <c r="C11" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D11" s="3">
         <v>46146</v>
       </c>
-      <c r="E11" s="7">
+      <c r="E11" s="3">
         <v>46149</v>
       </c>
-      <c r="F11" s="6" t="str">
+      <c r="F11" s="1" t="str">
         <f t="shared" si="0"/>
         <v>Concluído</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" s="5" t="s">
+      <c r="A12" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="B12" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C12" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="D12" s="7">
+      <c r="C12" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D12" s="3">
         <v>46146</v>
       </c>
-      <c r="E12" s="7">
+      <c r="E12" s="3">
         <v>46148</v>
       </c>
-      <c r="F12" s="6" t="str">
+      <c r="F12" s="1" t="str">
         <f t="shared" si="0"/>
         <v>Concluído</v>
       </c>
@@ -1393,12 +1384,12 @@
       <c r="D43" s="3">
         <v>46199</v>
       </c>
-      <c r="E43" s="1" t="s">
-        <v>34</v>
+      <c r="E43" s="3">
+        <v>46212</v>
       </c>
       <c r="F43" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>Pendente</v>
+        <v>Concluído</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
@@ -1414,12 +1405,12 @@
       <c r="D44" s="3">
         <v>46199</v>
       </c>
-      <c r="E44" s="1" t="s">
-        <v>34</v>
+      <c r="E44" s="3">
+        <v>46212</v>
       </c>
       <c r="F44" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>Pendente</v>
+        <v>Concluído</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">

</xml_diff>